<commit_message>
Rebuild the raw-data workbook with the eq. (3) columns and the Supplementary Fig. 1 sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1WQ3WGcJw8tT3QK2n57xo
</commit_message>
<xml_diff>
--- a/figures/update/figure_update_rawdata.xlsx
+++ b/figures/update/figure_update_rawdata.xlsx
@@ -12,12 +12,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2d" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2e" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2f" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3a_kITO" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3a_nAg" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5c" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5d" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5d_reference_lines" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_Table1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_Fig1_nsub" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3a_kITO" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3a_nAg" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5c" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5d" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5d_reference_lines" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_Table1" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -447,7 +448,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>every eta_ext / EQE below is the matrix series of eq. (1) with the hemispherical MLA BSDF (n_MLA = n_sub); p is the cos.sin-weighted B_T of the structure</t>
+          <t>Fig. 2(c)-(f): closed form eq. (3), eta_ext = p / [p + (1 - p) A'], with p the cos.sin-weighted B_T of the hemispherical MLA (n_MLA = n_sub) and A' the cos.sin-weighted 1 - R_LED.  Fig. 3(a), 5(c), 5(d), SI Table 1: matrix series of eq. (1).  Decision of 2026-09-22: the series shows mode cut-off steps against n_sub (SI_Fig1_nsub), so the trend panels of Fig. 2 use eq. (3).</t>
         </is>
       </c>
     </row>
@@ -462,7 +463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eta_ext vs ITO thickness, n_sub 1.5, Al and Ag.  Was eq. (3) with p = 0.38.  Not monotonic any more (Ag 0.91 / 0.95 / 0.94 / 0.91 at 50 / 100 / 150 / 200 nm); Ag above Al by 12-15 %p everywhere.</t>
+          <t>eta_ext vs ITO thickness, n_sub 1.5, eq. (3) with p = 0.427.  Ag 0.969 (30 nm) -&gt; 0.933 (200 nm), Al 0.843 -&gt; 0.822; Ag above Al by 11-13 %p.  Measured green device 0.916 at 150 nm ITO for reference.</t>
         </is>
       </c>
     </row>
@@ -486,7 +487,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>eta_ext vs n_sub, series.  Gap Ag - Al: 7 %p (1.3), 13 %p (1.5), 21 %p (2.0).</t>
+          <t>eta_ext vs n_sub, eq. (3).  Gap Ag - Al: 7 %p (1.3), 12 %p (1.5), 22 %p (2.0).  Smooth; the series version with its cut-off dips is in SI_Fig1_nsub.</t>
         </is>
       </c>
     </row>
@@ -498,116 +499,128 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>eta_sub (unchanged) and EQE vs n_sub, series; extraction loss = eta_sub - EQE.  Al plateaus at 55-59 % for n &gt;= 1.8 (was a 63 % maximum); Ag 84 % at 1.8, 87 % at 2.0 (was 89 %).</t>
+          <t>eta_sub (unchanged) and EQE vs n_sub, eq. (3); extraction loss = eta_sub - EQE.  Al 61 % maximum at 1.8 then 58-60 %; Ag 89 % at 1.8, 87 % at 2.0.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Fig. 2(a),(b),(g)-(j)</t>
+          <t>SI_Fig1_nsub</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>unchanged (A' split and the angle/wavelength maps do not depend on the extraction model).</t>
+          <t>Supplementary Fig. 1 data: same stack, n_sub in 0.01 steps (BSDF interpolated between the 0.05 slices): eta_ext and EQE by eq. (3) and by the series, P_sub fraction beyond 70 deg.  Guided modes at 550 nm: n_eff 1.352 (TM), 1.523 (TE), 1.663 (TM), 1.734 (TE).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Fig. 3(a)</t>
+          <t>Fig. 2(a),(b),(g)-(j)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>k_ITO and n_Ag sweeps at n_sub 1.8, series.  k 0 -&gt; 0.01: eta_ext 0.95 -&gt; 0.81, EQE 0.91 -&gt; 0.75 (was 0.96 -&gt; 0.88, 0.93 -&gt; 0.82); k 0.08: EQE 0.45 (was 0.49).  n_Ag 0.2: EQE 0.55 (was 0.60).</t>
+          <t>unchanged (A' split and the angle/wavelength maps do not depend on the extraction model).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Fig. 3(b),(c)</t>
+          <t>Fig. 3(a)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>unchanged.</t>
+          <t>k_ITO and n_Ag sweeps at n_sub 1.8, series.  k 0 -&gt; 0.01: eta_ext 0.95 -&gt; 0.81, EQE 0.91 -&gt; 0.75 (was 0.96 -&gt; 0.88, 0.93 -&gt; 0.82); k 0.08: EQE 0.45 (was 0.49).  n_Ag 0.2: EQE 0.55 (was 0.60).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Fig. 5(c)</t>
+          <t>Fig. 3(b),(c)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EQE vs Theta, series.  proposed 83.1 -&gt; 85.0 % (was 88.4 -&gt; 91.2), reference 31.3 -&gt; 54.8 % (was 34 -&gt; 60).</t>
+          <t>unchanged.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Fig. 5(d)</t>
+          <t>Fig. 5(c)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>new panel: EQE vs lens aspect ratio, n_sub = n_MLA 1.8, close-packed hexagonal, series.  Ag max 86.6 % at AR 0.55, &gt;= 95 % of it for AR 0.25-1.5; Al max 56.2 % at 0.6, from 0.35.  Flat interface 25.5 / 21.6 %.  The AR = 1 row equals the LightTools slice-11 hemisphere.</t>
+          <t>EQE vs Theta, series.  proposed 83.1 -&gt; 85.0 % (was 88.4 -&gt; 91.2), reference 31.3 -&gt; 54.8 % (was 34 -&gt; 60).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Fig. 5(a),(b),(e), Fig. 4</t>
+          <t>Fig. 5(d)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>unchanged (author's series data).</t>
+          <t>new panel: EQE vs lens aspect ratio, n_sub = n_MLA 1.8, close-packed hexagonal, series.  Ag max 86.6 % at AR 0.55, &gt;= 95 % of it for AR 0.25-1.5; Al max 56.2 % at 0.6, from 0.35.  Flat interface 25.5 / 21.6 %.  The AR = 1 row equals the LightTools slice-11 hemisphere.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>Fig. 5(a),(b),(e), Fig. 4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>unchanged (author's series data).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
           <t>SI Table 1</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>real material stack, series: 87 % isotropic, 87.5-88 % at Theta 0.8-0.9, 89-90 % with k_ITO 0.002.  Eq. (3) values in brackets for reference.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n"/>
-    </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Stack</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>air | reflector 100 nm | ETL 1.8 | EML 1.8 20 nm | HTL 1.8 | ITO (Koenig 2014) | n_sub; 550 nm, PLQY 1, Theta 2/3 unless swept; Ag McPeak, Al Johnson-Christy type.  Fig. 2(d)-(f) and 3(a): ITO 50 nm; Fig. 2(c): ITO swept; Fig. 5(c) reference: Al, n 1.5, ETL/HTL 80/230; proposed: Ag, n 1.8, 200/200.</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>air | reflector 100 nm | ETL 1.8 | EML 1.8 20 nm | HTL 1.8 | ITO (Koenig 2014) | n_sub; 550 nm, PLQY 1, Theta 2/3 unless swept; Ag McPeak, Al Johnson-Christy type.  Fig. 2(d)-(f) and 3(a): ITO 50 nm; Fig. 2(c): ITO swept; Fig. 5(c) reference: Al, n 1.5, ETL/HTL 80/230; proposed: Ag, n 1.8, 200/200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>sim/audit/recompute_series.py, sim/mla/run_aspect.py; repository jjoono/OLED-, branch claude/oled-efficiency-paper-ag-955zsk</t>
         </is>
@@ -619,6 +632,605 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>aspect_ratio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>p_single_pass</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>EQE_Al</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>EQE_Ag</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>lens_shape</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.26928</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.327257</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.644772</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.270897</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.399737</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.7446159999999999</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.272682</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.456681</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.7977880000000001</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.274359</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.497019</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.827919</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.275978</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.523707</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.845338</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.277609</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.540156</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.855079</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.279087</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.549727</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.860253</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.280436</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.555524</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.863171</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.281869</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.559381</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.8649559999999999</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.283096</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.56142</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.865543</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.284205</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.561527</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.864577</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0.28519</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.5597220000000001</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.861737</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0.286052</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.556945</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.857471</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0.286687</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0.554359</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.85234</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0.287285</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0.552556</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.846868</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0.287752</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>0.552074</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0.842102</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0.288078</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.552812</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.838966</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0.288138</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0.554097</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.837647</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0.288424</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0.555115</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.837104</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0.28909</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>0.555412</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0.835975</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0.289453</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>0.555242</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0.835323</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0.289852</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>0.55427</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.834748</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0.290285</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>0.55266</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.834191</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0.290691</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>0.550553</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0.833175</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0.29117</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0.548252</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0.831968</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0.29151</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>0.54592</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>0.830909</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0.291913</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0.543689</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0.829875</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0.292271</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>0.541509</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>0.828728</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0.292603</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0.539447</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>0.82765</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ellipsoid</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -680,7 +1292,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1193,13 +1805,13 @@
         <v>0.139156</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.804172</v>
+        <v>0.842851</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0.023887</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.945065</v>
+        <v>0.968987</v>
       </c>
     </row>
     <row r="3">
@@ -1210,13 +1822,13 @@
         <v>0.140725</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.793927</v>
+        <v>0.841361</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0.025711</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.931178</v>
+        <v>0.966699</v>
       </c>
     </row>
     <row r="4">
@@ -1227,13 +1839,13 @@
         <v>0.142582</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.781984</v>
+        <v>0.839603</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>0.02755</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.911254</v>
+        <v>0.964401</v>
       </c>
     </row>
     <row r="5">
@@ -1244,13 +1856,13 @@
         <v>0.144739</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.769609</v>
+        <v>0.83757</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0.029072</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.894604</v>
+        <v>0.962508</v>
       </c>
     </row>
     <row r="6">
@@ -1261,13 +1873,13 @@
         <v>0.146999</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.759393</v>
+        <v>0.8354510000000001</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.028951</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.933082</v>
+        <v>0.962658</v>
       </c>
     </row>
     <row r="7">
@@ -1278,13 +1890,13 @@
         <v>0.148292</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.758841</v>
+        <v>0.834244</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0.029697</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.947926</v>
+        <v>0.9617329999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1295,13 +1907,13 @@
         <v>0.146725</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.780013</v>
+        <v>0.835708</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0.031059</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.952923</v>
+        <v>0.960048</v>
       </c>
     </row>
     <row r="9">
@@ -1312,13 +1924,13 @@
         <v>0.145833</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.800233</v>
+        <v>0.836543</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0.032819</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.953784</v>
+        <v>0.957879</v>
       </c>
     </row>
     <row r="10">
@@ -1329,13 +1941,13 @@
         <v>0.146576</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.811155</v>
+        <v>0.835847</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.034799</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.952715</v>
+        <v>0.955452</v>
       </c>
     </row>
     <row r="11">
@@ -1346,13 +1958,13 @@
         <v>0.148129</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.81619</v>
+        <v>0.834396</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>0.036859</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.950709</v>
+        <v>0.952939</v>
       </c>
     </row>
     <row r="12">
@@ -1363,13 +1975,13 @@
         <v>0.149877</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.818092</v>
+        <v>0.832768</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0.038915</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.948182</v>
+        <v>0.950443</v>
       </c>
     </row>
     <row r="13">
@@ -1380,13 +1992,13 @@
         <v>0.15153</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.818201</v>
+        <v>0.831236</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0.040934</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.945233</v>
+        <v>0.948005</v>
       </c>
     </row>
     <row r="14">
@@ -1397,13 +2009,13 @@
         <v>0.153022</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.816968</v>
+        <v>0.829856</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0.042917</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.94179</v>
+        <v>0.945624</v>
       </c>
     </row>
     <row r="15">
@@ -1414,13 +2026,13 @@
         <v>0.154409</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.814422</v>
+        <v>0.828578</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0.044884</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.937696</v>
+        <v>0.943273</v>
       </c>
     </row>
     <row r="16">
@@ -1431,13 +2043,13 @@
         <v>0.155798</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.810437</v>
+        <v>0.827302</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0.046867</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.93275</v>
+        <v>0.9409149999999999</v>
       </c>
     </row>
     <row r="17">
@@ -1448,13 +2060,13 @@
         <v>0.157316</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0.804878</v>
+        <v>0.825913</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0.048907</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.9267339999999999</v>
+        <v>0.938501</v>
       </c>
     </row>
     <row r="18">
@@ -1465,13 +2077,13 @@
         <v>0.159093</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.797667</v>
+        <v>0.824292</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0.05105</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.919426</v>
+        <v>0.935979</v>
       </c>
     </row>
     <row r="19">
@@ -1482,13 +2094,13 @@
         <v>0.161253</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0.788841</v>
+        <v>0.82233</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0.053343</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.910621</v>
+        <v>0.933295</v>
       </c>
     </row>
   </sheetData>
@@ -1784,10 +2396,10 @@
         <v>1.3</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.91625</v>
+        <v>0.915201</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.981425</v>
+        <v>0.982445</v>
       </c>
     </row>
     <row r="3">
@@ -1795,10 +2407,10 @@
         <v>1.35</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.896525</v>
+        <v>0.899375</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.9798289999999999</v>
+        <v>0.979414</v>
       </c>
     </row>
     <row r="4">
@@ -1806,10 +2418,10 @@
         <v>1.4</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.856164</v>
+        <v>0.880178</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.974759</v>
+        <v>0.975961</v>
       </c>
     </row>
     <row r="5">
@@ -1817,10 +2429,10 @@
         <v>1.45</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.782561</v>
+        <v>0.855059</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.957159</v>
+        <v>0.971162</v>
       </c>
     </row>
     <row r="6">
@@ -1828,10 +2440,10 @@
         <v>1.5</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.781984</v>
+        <v>0.839603</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.911254</v>
+        <v>0.964401</v>
       </c>
     </row>
     <row r="7">
@@ -1839,10 +2451,10 @@
         <v>1.55</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.77745</v>
+        <v>0.825288</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.931971</v>
+        <v>0.960934</v>
       </c>
     </row>
     <row r="8">
@@ -1850,10 +2462,10 @@
         <v>1.6</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.679673</v>
+        <v>0.803886</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.889701</v>
+        <v>0.953958</v>
       </c>
     </row>
     <row r="9">
@@ -1861,10 +2473,10 @@
         <v>1.65</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.700986</v>
+        <v>0.790141</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.902596</v>
+        <v>0.949512</v>
       </c>
     </row>
     <row r="10">
@@ -1872,10 +2484,10 @@
         <v>1.7</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.710217</v>
+        <v>0.775518</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.921121</v>
+        <v>0.946612</v>
       </c>
     </row>
     <row r="11">
@@ -1883,10 +2495,10 @@
         <v>1.75</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.689263</v>
+        <v>0.75334</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.917007</v>
+        <v>0.942232</v>
       </c>
     </row>
     <row r="12">
@@ -1894,10 +2506,10 @@
         <v>1.8</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.659498</v>
+        <v>0.730289</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.875528</v>
+        <v>0.929019</v>
       </c>
     </row>
     <row r="13">
@@ -1905,10 +2517,10 @@
         <v>1.85</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.693543</v>
+        <v>0.718946</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.906855</v>
+        <v>0.926107</v>
       </c>
     </row>
     <row r="14">
@@ -1916,10 +2528,10 @@
         <v>1.9</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.705654</v>
+        <v>0.706744</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.918532</v>
+        <v>0.923517</v>
       </c>
     </row>
     <row r="15">
@@ -1927,10 +2539,10 @@
         <v>1.95</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0.713441</v>
+        <v>0.701417</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.923052</v>
+        <v>0.9210429999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1938,10 +2550,10 @@
         <v>2</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.713407</v>
+        <v>0.696864</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.923548</v>
+        <v>0.9185990000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2012,19 +2624,19 @@
         <v>0.264561</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.242404</v>
+        <v>0.242126</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.02215699999999998</v>
+        <v>0.02243499999999998</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>0.313559</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.307735</v>
+        <v>0.308055</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.005823999999999996</v>
+        <v>0.005503999999999953</v>
       </c>
     </row>
     <row r="3">
@@ -2035,19 +2647,19 @@
         <v>0.284534</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.255092</v>
+        <v>0.255903</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.02944200000000002</v>
+        <v>0.02863100000000002</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>0.330255</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.323594</v>
+        <v>0.323457</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>0.006661000000000028</v>
+        <v>0.006798000000000026</v>
       </c>
     </row>
     <row r="4">
@@ -2058,19 +2670,19 @@
         <v>0.316716</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.271161</v>
+        <v>0.278767</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.04555500000000001</v>
+        <v>0.03794900000000001</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>0.353833</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.344902</v>
+        <v>0.345327</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.008931000000000022</v>
+        <v>0.008506000000000014</v>
       </c>
     </row>
     <row r="5">
@@ -2081,19 +2693,19 @@
         <v>0.371693</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.290872</v>
+        <v>0.317819</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.08082099999999998</v>
+        <v>0.05387399999999998</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0.396883</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.37988</v>
+        <v>0.385438</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.01700299999999999</v>
+        <v>0.01144499999999998</v>
       </c>
     </row>
     <row r="6">
@@ -2104,19 +2716,19 @@
         <v>0.396981</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.310433</v>
+        <v>0.333306</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.08654799999999996</v>
+        <v>0.06367499999999998</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0.474062</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.431991</v>
+        <v>0.457185</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.04207099999999997</v>
+        <v>0.01687699999999998</v>
       </c>
     </row>
     <row r="7">
@@ -2127,19 +2739,19 @@
         <v>0.425557</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.330849</v>
+        <v>0.351207</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.09470800000000001</v>
+        <v>0.07435000000000003</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>0.498066</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.464183</v>
+        <v>0.478609</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.033883</v>
+        <v>0.019457</v>
       </c>
     </row>
     <row r="8">
@@ -2150,19 +2762,19 @@
         <v>0.542357</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.368625</v>
+        <v>0.435993</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.173732</v>
+        <v>0.106364</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>0.58497</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.520448</v>
+        <v>0.558037</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.06452199999999997</v>
+        <v>0.02693299999999998</v>
       </c>
     </row>
     <row r="9">
@@ -2173,19 +2785,19 @@
         <v>0.59518</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.417213</v>
+        <v>0.470276</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.177967</v>
+        <v>0.124904</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>0.664357</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.599646</v>
+        <v>0.630815</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.06471099999999996</v>
+        <v>0.03354199999999996</v>
       </c>
     </row>
     <row r="10">
@@ -2196,19 +2808,19 @@
         <v>0.646443</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.459115</v>
+        <v>0.501328</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.187328</v>
+        <v>0.145115</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0.718771</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.662076</v>
+        <v>0.680397</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.05669500000000005</v>
+        <v>0.03837400000000002</v>
       </c>
     </row>
     <row r="11">
@@ -2219,19 +2831,19 @@
         <v>0.72784</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.501673</v>
+        <v>0.548311</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.226167</v>
+        <v>0.179529</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>0.812313</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.744897</v>
+        <v>0.765387</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.06741599999999992</v>
+        <v>0.04692599999999991</v>
       </c>
     </row>
     <row r="12">
@@ -2242,19 +2854,19 @@
         <v>0.8414779999999999</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.554953</v>
+        <v>0.614523</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.2865249999999999</v>
+        <v>0.2269549999999999</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0.956185</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.837167</v>
+        <v>0.888314</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.119018</v>
+        <v>0.0678709999999999</v>
       </c>
     </row>
     <row r="13">
@@ -2265,19 +2877,19 @@
         <v>0.828731</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.574761</v>
+        <v>0.595813</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.25397</v>
+        <v>0.232918</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0.9388300000000001</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.851382</v>
+        <v>0.869456</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0.08744800000000008</v>
+        <v>0.06937400000000005</v>
       </c>
     </row>
     <row r="14">
@@ -2288,19 +2900,19 @@
         <v>0.829345</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.58523</v>
+        <v>0.586135</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.244115</v>
+        <v>0.24321</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>0.939436</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.8629019999999999</v>
+        <v>0.867586</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.0765340000000001</v>
+        <v>0.07185000000000008</v>
       </c>
     </row>
     <row r="15">
@@ -2311,19 +2923,19 @@
         <v>0.8304820000000001</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.5925010000000001</v>
+        <v>0.582515</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.237981</v>
+        <v>0.247967</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0.9409459999999999</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.868542</v>
+        <v>0.8666509999999999</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.07240399999999991</v>
+        <v>0.074295</v>
       </c>
     </row>
     <row r="16">
@@ -2334,19 +2946,19 @@
         <v>0.831483</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.593186</v>
+        <v>0.579431</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.238297</v>
+        <v>0.2520519999999999</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>0.942373</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.870327</v>
+        <v>0.865663</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.07204600000000005</v>
+        <v>0.07671000000000006</v>
       </c>
     </row>
   </sheetData>
@@ -2355,6 +2967,2575 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K72"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>n_sub</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext_eq3_Al</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext_series_Al</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>EQE_eq3_Al</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>EQE_series_Al</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Psub_beyond70deg_Al</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext_eq3_Ag</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext_series_Ag</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>EQE_eq3_Ag</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>EQE_series_Ag</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Psub_beyond70deg_Ag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.915201</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.91625</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.242126</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.242404</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.045367</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.982445</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.981425</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.308055</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.307735</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.039297</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.912314</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.9133829999999999</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.244519</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.244806</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.04747</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.981858</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.9813539999999999</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.310829</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.310669</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>0.038654</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.909303</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.910033</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.247062</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.24726</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.050196</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.9813</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.981179</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.313745</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.313707</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0.038676</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.906156</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.906156</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.249783</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.249783</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.053591</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.980696</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.980857</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.316802</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0.316854</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>0.039297</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.902854</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.901685</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.252716</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.252388</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.057725</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.9800450000000001</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.980392</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.320022</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0.320135</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.040494</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.899375</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.896525</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.255903</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.255092</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.062699</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.979414</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.9798289999999999</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0.323457</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0.323594</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>0.042256</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.896048</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.890917</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.259501</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.258015</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.06865</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.978762</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.979165</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0.32713</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0.327265</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0.044619</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.892508</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.884344</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.263485</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.261075</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0.075754</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0.978154</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0.978399</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0.33111</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0.331193</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>0.047625</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.888717</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.8765770000000001</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.267943</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.264283</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.08423899999999999</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.977453</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.977416</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0.335407</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0.335394</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0.051366</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.8846270000000001</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.8673110000000001</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.272989</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.267646</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>0.094389</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0.976733</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>0.976229</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>0.340118</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0.339942</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>0.055953</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.880178</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.856164</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.278767</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.271161</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.106547</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.975961</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0.974759</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.345327</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0.344902</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0.061556</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0.87566</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.843065</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.285567</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.274937</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0.121081</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0.975162</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0.972965</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.35117</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0.350379</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>0.068395</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0.8706700000000001</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.827329</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.29345</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.278843</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.138224</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.974369</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.970705</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.357832</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.356486</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0.076776</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0.865225</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0.809324</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.302371</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0.282836</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0.157437</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0.973202</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0.967471</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.365412</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0.36326</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0.087132</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0.859721</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0.792266</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.311277</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0.286854</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.175214</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.972411</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.963406</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.374542</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0.371074</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0.100032</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0.855059</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>0.782561</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0.317819</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0.290872</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0.184742</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0.971162</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.957159</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.385438</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0.37988</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0.116365</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0.851568</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.7796110000000001</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.322184</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.29496</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.186904</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.969915</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.947731</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.399112</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0.389983</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0.137361</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0.848449</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0.779385</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.325454</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0.298962</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0.185481</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0.968359</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0.932154</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0.416788</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0.401205</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0.164845</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0.845477</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0.780164</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.328226</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0.30287</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.182247</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.966154</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0.906393</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0.439687</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0.41249</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0.200174</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0.842549</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>0.7811669999999999</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0.330786</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0.306688</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0.178051</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0.9651459999999999</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>0.902214</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0.452815</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0.42329</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0.21316</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0.839603</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>0.781984</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0.333306</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.310433</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.17341</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.964401</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0.911254</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0.457185</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0.431991</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0.210143</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0.836961</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>0.782775</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.336062</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0.314305</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>0.168731</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>0.963734</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0.918614</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>0.460914</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>0.439335</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>0.205453</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0.834242</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>0.78295</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.339045</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0.318199</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>0.164408</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>0.963152</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0.924104</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>0.464711</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>0.44587</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>0.200278</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0.831416</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>0.782311</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0.342407</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>0.322183</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>0.16089</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>0.962426</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>0.927941</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>0.468736</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>0.451941</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>0.195093</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0.828446</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0.780606</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0.346355</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>0.326354</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0.158751</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>0.9617019999999999</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0.930536</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>0.473284</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>0.457946</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>0.190271</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0.825288</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>0.77745</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>0.351207</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>0.330849</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>0.1588</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>0.960934</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>0.931971</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>0.478609</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>0.464183</v>
+      </c>
+      <c r="K27" s="3" t="n">
+        <v>0.186321</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0.822192</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0.772581</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0.357633</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>0.336054</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>0.162283</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>0.960057</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0.932266</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>0.4851</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>0.471059</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>0.183972</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0.818743</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>0.764247</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>0.366497</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>0.342103</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>0.171339</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>0.959103</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>0.931016</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>0.493507</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>0.479055</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>0.184399</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0.814733</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0.749382</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>0.379886</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>0.349415</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0.190055</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>0.95797</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>0.9271779999999999</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>0.505221</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>0.488981</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <v>0.189829</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0.809713</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>0.720388</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0.402811</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>0.358374</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0.226955</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>0.956396</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>0.917513</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>0.523465</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>0.502183</v>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v>0.204987</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0.803886</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>0.679673</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>0.435993</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>0.368625</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0.277841</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>0.953958</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0.889701</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>0.558037</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>0.520448</v>
+      </c>
+      <c r="K32" s="3" t="n">
+        <v>0.242259</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0.800794</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>0.678832</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0.447644</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>0.379467</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>0.285762</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>0.951751</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>0.861538</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>0.598538</v>
+      </c>
+      <c r="J33" s="3" t="n">
+        <v>0.541805</v>
+      </c>
+      <c r="K33" s="3" t="n">
+        <v>0.281783</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0.798159</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>0.684737</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0.454245</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0.389695</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>0.284516</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>0.951128</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>0.875822</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>0.607681</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>0.559568</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>0.279346</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0.795557</v>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>0.69093</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>0.459796</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>0.399326</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>0.280809</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>0.949978</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>0.886616</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>0.614924</v>
+      </c>
+      <c r="J35" s="3" t="n">
+        <v>0.57391</v>
+      </c>
+      <c r="K35" s="3" t="n">
+        <v>0.274593</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0.792898</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>0.696427</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>0.465046</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>0.408464</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>0.275764</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>0.950035</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>0.895772</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>0.622903</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>0.587325</v>
+      </c>
+      <c r="K36" s="3" t="n">
+        <v>0.269087</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0.790141</v>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>0.700986</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>0.470276</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>0.417213</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>0.269709</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>0.949512</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>0.902596</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>0.630815</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>0.599646</v>
+      </c>
+      <c r="K37" s="3" t="n">
+        <v>0.263204</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0.787578</v>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>0.704986</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>0.475831</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>0.425932</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0.262787</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>0.948997</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>0.908214</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>0.63922</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>0.61175</v>
+      </c>
+      <c r="K38" s="3" t="n">
+        <v>0.256965</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0.784869</v>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>0.707937</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>0.48163</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>0.434422</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>0.255142</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>0.948478</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>0.912737</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>0.648253</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>0.623825</v>
+      </c>
+      <c r="K39" s="3" t="n">
+        <v>0.250379</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0.781982</v>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>0.7098179999999999</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>0.487758</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0.442746</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0.246993</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>0.948034</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>0.916429</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>0.658107</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>0.636167</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>0.24354</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0.778881</v>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>0.710596</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>0.494297</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>0.450961</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>0.238679</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>0.947488</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>0.9192669999999999</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>0.668816</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>0.648895</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>0.236631</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0.775518</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>0.710217</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>0.501328</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>0.459115</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>0.230651</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>0.946612</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>0.921121</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>0.680397</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>0.662076</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>0.229981</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0.77212</v>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>0.708919</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>0.509132</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>0.467458</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>0.223425</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>0.946232</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>0.922749</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>0.693671</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>0.6764559999999999</v>
+      </c>
+      <c r="K43" s="3" t="n">
+        <v>0.22397</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0.768327</v>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>0.706281</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>0.51763</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>0.475829</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>0.217521</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>0.945576</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>0.923374</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>0.708368</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>0.691736</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>0.219173</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0.764031</v>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>0.702179</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>0.526926</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>0.484269</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0.213399</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>0.94474</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>0.922921</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>0.72492</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>0.7081769999999999</v>
+      </c>
+      <c r="K45" s="3" t="n">
+        <v>0.216112</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0.759087</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>0.696508</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>0.537125</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>0.492844</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>0.211426</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>0.943361</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>0.920764</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>0.743511</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>0.725702</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>0.21533</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0.75334</v>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>0.689263</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>0.548311</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>0.501673</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>0.211827</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>0.942232</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>0.917007</v>
+      </c>
+      <c r="I47" s="3" t="n">
+        <v>0.765387</v>
+      </c>
+      <c r="J47" s="3" t="n">
+        <v>0.744897</v>
+      </c>
+      <c r="K47" s="3" t="n">
+        <v>0.217276</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0.747126</v>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>0.681049</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>0.560768</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>0.511173</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>0.214489</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>0.940437</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>0.909964</v>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>0.790631</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>0.765012</v>
+      </c>
+      <c r="K48" s="3" t="n">
+        <v>0.222502</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0.741462</v>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>0.672925</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>0.574567</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>0.5214569999999999</v>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>0.218179</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>0.937747</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>0.898146</v>
+      </c>
+      <c r="I49" s="3" t="n">
+        <v>0.819986</v>
+      </c>
+      <c r="J49" s="3" t="n">
+        <v>0.785358</v>
+      </c>
+      <c r="K49" s="3" t="n">
+        <v>0.231415</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0.737339</v>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>0.664842</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>0.590846</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>0.532753</v>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>0.223036</v>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>0.933805</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>0.881566</v>
+      </c>
+      <c r="I50" s="3" t="n">
+        <v>0.852447</v>
+      </c>
+      <c r="J50" s="3" t="n">
+        <v>0.804759</v>
+      </c>
+      <c r="K50" s="3" t="n">
+        <v>0.243007</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0.733215</v>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>0.654819</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>0.609648</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>0.5444639999999999</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>0.230458</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>0.930661</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>0.871213</v>
+      </c>
+      <c r="I51" s="3" t="n">
+        <v>0.879233</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>0.82307</v>
+      </c>
+      <c r="K51" s="3" t="n">
+        <v>0.247146</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0.730289</v>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>0.659498</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>0.614523</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>0.554953</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>0.217914</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>0.929019</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>0.875528</v>
+      </c>
+      <c r="I52" s="3" t="n">
+        <v>0.888314</v>
+      </c>
+      <c r="J52" s="3" t="n">
+        <v>0.837167</v>
+      </c>
+      <c r="K52" s="3" t="n">
+        <v>0.233926</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0.728253</v>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>0.668708</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>0.606936</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>0.55731</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>0.196734</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>0.928399</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>0.884888</v>
+      </c>
+      <c r="I53" s="3" t="n">
+        <v>0.877918</v>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>0.836772</v>
+      </c>
+      <c r="K53" s="3" t="n">
+        <v>0.211664</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0.7262</v>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>0.676724</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>0.60326</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>0.56216</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>0.174001</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>0.9278189999999999</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>0.8922870000000001</v>
+      </c>
+      <c r="I54" s="3" t="n">
+        <v>0.873841</v>
+      </c>
+      <c r="J54" s="3" t="n">
+        <v>0.840377</v>
+      </c>
+      <c r="K54" s="3" t="n">
+        <v>0.187696</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>0.724028</v>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>0.683503</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>0.600584</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>0.566968</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>0.150377</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>0.926256</v>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>0.897388</v>
+      </c>
+      <c r="I55" s="3" t="n">
+        <v>0.870738</v>
+      </c>
+      <c r="J55" s="3" t="n">
+        <v>0.843601</v>
+      </c>
+      <c r="K55" s="3" t="n">
+        <v>0.162647</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0.721647</v>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>0.689101</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>0.598208</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>0.571229</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>0.126609</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>0.9266529999999999</v>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>0.902935</v>
+      </c>
+      <c r="I56" s="3" t="n">
+        <v>0.870319</v>
+      </c>
+      <c r="J56" s="3" t="n">
+        <v>0.848043</v>
+      </c>
+      <c r="K56" s="3" t="n">
+        <v>0.137167</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0.718946</v>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>0.693543</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>0.595813</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>0.574761</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>0.103819</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>0.926107</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>0.906855</v>
+      </c>
+      <c r="I57" s="3" t="n">
+        <v>0.869456</v>
+      </c>
+      <c r="J57" s="3" t="n">
+        <v>0.851382</v>
+      </c>
+      <c r="K57" s="3" t="n">
+        <v>0.112386</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>0.716117</v>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>0.697065</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>0.593449</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>0.57766</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>0.083385</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>0.925623</v>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>0.910137</v>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>0.868904</v>
+      </c>
+      <c r="J58" s="3" t="n">
+        <v>0.854367</v>
+      </c>
+      <c r="K58" s="3" t="n">
+        <v>0.08956</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="B59" s="3" t="n">
+        <v>0.713106</v>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>0.6996019999999999</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>0.591014</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>0.5798219999999999</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>0.066395</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>0.9250969999999999</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>0.912838</v>
+      </c>
+      <c r="I59" s="3" t="n">
+        <v>0.868466</v>
+      </c>
+      <c r="J59" s="3" t="n">
+        <v>0.856957</v>
+      </c>
+      <c r="K59" s="3" t="n">
+        <v>0.06979100000000001</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="B60" s="3" t="n">
+        <v>0.71047</v>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>0.701669</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>0.588936</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>0.581641</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>0.052954</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>0.924226</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>0.914806</v>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>0.867798</v>
+      </c>
+      <c r="J60" s="3" t="n">
+        <v>0.858953</v>
+      </c>
+      <c r="K60" s="3" t="n">
+        <v>0.05362</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="B61" s="3" t="n">
+        <v>0.708407</v>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>0.703674</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>0.5873620000000001</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>0.583438</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>0.042558</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>0.924038</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>0.916965</v>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>0.86783</v>
+      </c>
+      <c r="J61" s="3" t="n">
+        <v>0.861187</v>
+      </c>
+      <c r="K61" s="3" t="n">
+        <v>0.040955</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="B62" s="3" t="n">
+        <v>0.706744</v>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>0.705654</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>0.586135</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>0.58523</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>0.034664</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>0.923517</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>0.918532</v>
+      </c>
+      <c r="I62" s="3" t="n">
+        <v>0.867586</v>
+      </c>
+      <c r="J62" s="3" t="n">
+        <v>0.8629019999999999</v>
+      </c>
+      <c r="K62" s="3" t="n">
+        <v>0.031309</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="B63" s="3" t="n">
+        <v>0.705568</v>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>0.70778</v>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>0.585319</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>0.587154</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>0.028742</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>0.923059</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>0.919894</v>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>0.867421</v>
+      </c>
+      <c r="J63" s="3" t="n">
+        <v>0.864447</v>
+      </c>
+      <c r="K63" s="3" t="n">
+        <v>0.024058</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="B64" s="3" t="n">
+        <v>0.7045</v>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>0.7096789999999999</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>0.584596</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>0.588893</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>0.02431</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>0.922566</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>0.9209889999999999</v>
+      </c>
+      <c r="I64" s="3" t="n">
+        <v>0.867236</v>
+      </c>
+      <c r="J64" s="3" t="n">
+        <v>0.865754</v>
+      </c>
+      <c r="K64" s="3" t="n">
+        <v>0.018627</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="B65" s="3" t="n">
+        <v>0.703475</v>
+      </c>
+      <c r="C65" s="3" t="n">
+        <v>0.71128</v>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>0.583907</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>0.590386</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>0.020964</v>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>0.921346</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>0.921251</v>
+      </c>
+      <c r="I65" s="3" t="n">
+        <v>0.8663729999999999</v>
+      </c>
+      <c r="J65" s="3" t="n">
+        <v>0.866283</v>
+      </c>
+      <c r="K65" s="3" t="n">
+        <v>0.014547</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="B66" s="3" t="n">
+        <v>0.702454</v>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>0.712542</v>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>0.58322</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>0.591595</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0.018384</v>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>0.921535</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>0.922529</v>
+      </c>
+      <c r="I66" s="3" t="n">
+        <v>0.866834</v>
+      </c>
+      <c r="J66" s="3" t="n">
+        <v>0.867769</v>
+      </c>
+      <c r="K66" s="3" t="n">
+        <v>0.011461</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="B67" s="3" t="n">
+        <v>0.701417</v>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>0.713441</v>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>0.582515</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>0.5925010000000001</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>0.016309</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>0.9210429999999999</v>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>0.923052</v>
+      </c>
+      <c r="I67" s="3" t="n">
+        <v>0.8666509999999999</v>
+      </c>
+      <c r="J67" s="3" t="n">
+        <v>0.868542</v>
+      </c>
+      <c r="K67" s="3" t="n">
+        <v>0.009109000000000001</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="B68" s="3" t="n">
+        <v>0.700582</v>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>0.714191</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>0.581972</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>0.5932770000000001</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>0.014499</v>
+      </c>
+      <c r="G68" s="3" t="n">
+        <v>0.9205950000000001</v>
+      </c>
+      <c r="H68" s="3" t="n">
+        <v>0.923462</v>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>0.866506</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>0.869205</v>
+      </c>
+      <c r="K68" s="3" t="n">
+        <v>0.007301</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="B69" s="3" t="n">
+        <v>0.699713</v>
+      </c>
+      <c r="C69" s="3" t="n">
+        <v>0.714566</v>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>0.581396</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>0.593737</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>0.012699</v>
+      </c>
+      <c r="G69" s="3" t="n">
+        <v>0.920126</v>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>0.9237069999999999</v>
+      </c>
+      <c r="I69" s="3" t="n">
+        <v>0.866335</v>
+      </c>
+      <c r="J69" s="3" t="n">
+        <v>0.869707</v>
+      </c>
+      <c r="K69" s="3" t="n">
+        <v>0.005897</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="B70" s="3" t="n">
+        <v>0.698806</v>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>0.714557</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>0.580783</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>0.593874</v>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>0.010644</v>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>0.919403</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>0.923589</v>
+      </c>
+      <c r="I70" s="3" t="n">
+        <v>0.865917</v>
+      </c>
+      <c r="J70" s="3" t="n">
+        <v>0.86986</v>
+      </c>
+      <c r="K70" s="3" t="n">
+        <v>0.004797</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="B71" s="3" t="n">
+        <v>0.6978569999999999</v>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>0.714166</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>0.580128</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>0.593686</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>0.008364</v>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>0.919029</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>0.9236529999999999</v>
+      </c>
+      <c r="I71" s="3" t="n">
+        <v>0.865821</v>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>0.870177</v>
+      </c>
+      <c r="K71" s="3" t="n">
+        <v>0.003927</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B72" s="3" t="n">
+        <v>0.696864</v>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>0.713407</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>0.579431</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>0.593186</v>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>0.006366</v>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>0.9185990000000001</v>
+      </c>
+      <c r="H72" s="3" t="n">
+        <v>0.923548</v>
+      </c>
+      <c r="I72" s="3" t="n">
+        <v>0.865663</v>
+      </c>
+      <c r="J72" s="3" t="n">
+        <v>0.870327</v>
+      </c>
+      <c r="K72" s="3" t="n">
+        <v>0.003235</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2634,7 +5815,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2970,7 +6151,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3203,603 +6384,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>aspect_ratio</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>p_single_pass</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>EQE_Al</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>EQE_Ag</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>lens_shape</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>0.26928</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0.327257</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0.644772</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>0.270897</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>0.399737</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0.7446159999999999</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>0.272682</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.456681</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0.7977880000000001</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>0.274359</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.497019</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0.827919</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>0.275978</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>0.523707</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>0.845338</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>0.277609</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>0.540156</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0.855079</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>0.279087</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>0.549727</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>0.860253</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>0.280436</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>0.555524</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>0.863171</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>0.281869</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>0.559381</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>0.8649559999999999</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>0.283096</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>0.56142</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>0.865543</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>0.284205</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>0.561527</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>0.864577</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>0.28519</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>0.5597220000000001</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>0.861737</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>0.286052</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>0.556945</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>0.857471</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>0.286687</v>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>0.554359</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>0.85234</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>0.287285</v>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>0.552556</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>0.846868</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>0.287752</v>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>0.552074</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>0.842102</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>0.288078</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>0.552812</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>0.838966</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>0.288138</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>0.554097</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>0.837647</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>0.288424</v>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>0.555115</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>0.837104</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>0.28909</v>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>0.555412</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>0.835975</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>0.289453</v>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>0.555242</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>0.835323</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>0.289852</v>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>0.55427</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>0.834748</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="B24" s="3" t="n">
-        <v>0.290285</v>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>0.55266</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>0.834191</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="B25" s="3" t="n">
-        <v>0.290691</v>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>0.550553</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>0.833175</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="B26" s="3" t="n">
-        <v>0.29117</v>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>0.548252</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>0.831968</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="B27" s="3" t="n">
-        <v>0.29151</v>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>0.54592</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>0.830909</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="B28" s="3" t="n">
-        <v>0.291913</v>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>0.543689</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>0.829875</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="B29" s="3" t="n">
-        <v>0.292271</v>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>0.541509</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>0.828728</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>0.292603</v>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>0.539447</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>0.82765</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ellipsoid</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Substrate tunnelling booked to the substrate channel: Fig. 2(d)-(f) above n_sub 1.8 and Table 1 recomputed; Fig. 5 calculation conditions and deposition details in Methods
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1WQ3WGcJw8tT3QK2n57xo
</commit_message>
<xml_diff>
--- a/figures/update/figure_update_rawdata.xlsx
+++ b/figures/update/figure_update_rawdata.xlsx
@@ -499,7 +499,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>eta_sub (unchanged) and EQE vs n_sub, eq. (3); extraction loss = eta_sub - EQE.  Al 61 % maximum at 1.8 then 58-60 %; Ag 89 % at 1.8, 87 % at 2.0.</t>
+          <t>eta_sub and EQE vs n_sub, eq. (3); extraction loss = eta_sub - EQE.  Al 61 % maximum at 1.8 then 59-61 %; Ag 89 % at 1.8, 88 % at 2.0.  eta_sub for n_sub &gt; 1.8 now includes the near field that tunnels into the denser substrate (about 2 %p; it was booked as SPP before 2026-09-22).</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>real material stack, series: 87 % isotropic, 87.5-88 % at Theta 0.8-0.9, 89-90 % with k_ITO 0.002.  Eq. (3) values in brackets for reference.</t>
+          <t>real material stack, series: 88-89 % isotropic (ETL 200-300 nm), 88-89 % at Theta 0.8-0.9, 90-91 % with k_ITO 0.002.  Eq. (3) values alongside for reference.  Substrate tunnelling of the p-polarised near field (n_e,EML 1.67 &lt; n_sub 1.8) is included.</t>
         </is>
       </c>
     </row>
@@ -1376,10 +1376,10 @@
         <v>0.667</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.952339</v>
+        <v>0.9630649999999999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.033503</v>
+        <v>0.022777</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.029424</v>
@@ -1388,13 +1388,13 @@
         <v>0.912067</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.868597</v>
+        <v>0.87838</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0.932316</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.887881</v>
+        <v>0.897881</v>
       </c>
     </row>
     <row r="3">
@@ -1408,10 +1408,10 @@
         <v>0.8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.962929</v>
+        <v>0.970672</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.022878</v>
+        <v>0.015135</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.029424</v>
@@ -1420,13 +1420,13 @@
         <v>0.908308</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.874636</v>
+        <v>0.881669</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>0.932316</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.8977540000000001</v>
+        <v>0.904973</v>
       </c>
     </row>
     <row r="4">
@@ -1440,10 +1440,10 @@
         <v>0.9</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.970457</v>
+        <v>0.976079</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.015325</v>
+        <v>0.009703</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0.029424</v>
@@ -1452,13 +1452,13 @@
         <v>0.905671</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.878915</v>
+        <v>0.884007</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0.932316</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.904772</v>
+        <v>0.910014</v>
       </c>
     </row>
     <row r="5">
@@ -1472,10 +1472,10 @@
         <v>0.667</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.954833</v>
+        <v>0.965619</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.033498</v>
+        <v>0.022712</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0.024096</v>
@@ -1484,13 +1484,13 @@
         <v>0.929108</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.887143</v>
+        <v>0.897165</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>0.943885</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.901253</v>
+        <v>0.911433</v>
       </c>
     </row>
     <row r="6">
@@ -1504,10 +1504,10 @@
         <v>0.8</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.965516</v>
+        <v>0.973302</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.022869</v>
+        <v>0.015083</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0.024096</v>
@@ -1516,13 +1516,13 @@
         <v>0.926243</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.894302</v>
+        <v>0.901514</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0.943885</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.911336</v>
+        <v>0.918685</v>
       </c>
     </row>
     <row r="7">
@@ -1536,10 +1536,10 @@
         <v>0.9</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.9731109999999999</v>
+        <v>0.978764</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.015314</v>
+        <v>0.00966</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0.024096</v>
@@ -1548,13 +1548,13 @@
         <v>0.924233</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.899381</v>
+        <v>0.904606</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>0.943885</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.918504</v>
+        <v>0.923841</v>
       </c>
     </row>
     <row r="8">
@@ -1568,10 +1568,10 @@
         <v>0.667</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.962986</v>
+        <v>0.980537</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.020925</v>
+        <v>0.003373</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0.02893</v>
@@ -1580,13 +1580,13 @@
         <v>0.907432</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.873845</v>
+        <v>0.889772</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0.933376</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.898829</v>
+        <v>0.91521</v>
       </c>
     </row>
     <row r="9">
@@ -1600,10 +1600,10 @@
         <v>0.8</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.969566</v>
+        <v>0.981228</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.013945</v>
+        <v>0.002283</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0.02893</v>
@@ -1612,13 +1612,13 @@
         <v>0.9029239999999999</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.875444</v>
+        <v>0.885975</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>0.933376</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.904969</v>
+        <v>0.915855</v>
       </c>
     </row>
     <row r="10">
@@ -1632,10 +1632,10 @@
         <v>0.9</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.974371</v>
+        <v>0.981733</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.008847000000000001</v>
+        <v>0.001486</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0.02893</v>
@@ -1644,13 +1644,13 @@
         <v>0.899635</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.876578</v>
+        <v>0.883201</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>0.933376</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.909455</v>
+        <v>0.916326</v>
       </c>
     </row>
     <row r="11">
@@ -1664,10 +1664,10 @@
         <v>0.667</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.965882</v>
+        <v>0.983533</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.020925</v>
+        <v>0.003274</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0.023604</v>
@@ -1676,13 +1676,13 @@
         <v>0.9270119999999999</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.895384</v>
+        <v>0.911747</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>0.944968</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.912728</v>
+        <v>0.929408</v>
       </c>
     </row>
     <row r="12">
@@ -1696,10 +1696,10 @@
         <v>0.8</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.972601</v>
+        <v>0.98433</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.013938</v>
+        <v>0.002209</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0.023604</v>
@@ -1708,13 +1708,13 @@
         <v>0.9236220000000001</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.898315</v>
+        <v>0.909149</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>0.944968</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.919077</v>
+        <v>0.93016</v>
       </c>
     </row>
     <row r="13">
@@ -1728,10 +1728,10 @@
         <v>0.9</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.977508</v>
+        <v>0.984912</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.008835000000000001</v>
+        <v>0.001432</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>0.023604</v>
@@ -1740,13 +1740,13 @@
         <v>0.921149</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.900431</v>
+        <v>0.907251</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>0.944968</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.923714</v>
+        <v>0.93071</v>
       </c>
     </row>
   </sheetData>
@@ -2874,22 +2874,22 @@
         <v>1.85</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.828731</v>
+        <v>0.845467</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.595813</v>
+        <v>0.607845</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.232918</v>
+        <v>0.237622</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.9388300000000001</v>
+        <v>0.959183</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.869456</v>
+        <v>0.888306</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0.06937400000000005</v>
+        <v>0.07087699999999997</v>
       </c>
     </row>
     <row r="14">
@@ -2897,22 +2897,22 @@
         <v>1.9</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.829345</v>
+        <v>0.851217</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.586135</v>
+        <v>0.601593</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.24321</v>
+        <v>0.249624</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.939436</v>
+        <v>0.9598640000000001</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.867586</v>
+        <v>0.886451</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.07185000000000008</v>
+        <v>0.07341300000000006</v>
       </c>
     </row>
     <row r="15">
@@ -2920,22 +2920,22 @@
         <v>1.95</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0.8304820000000001</v>
+        <v>0.8527979999999999</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.582515</v>
+        <v>0.598167</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.247967</v>
+        <v>0.2546309999999999</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.9409459999999999</v>
+        <v>0.960224</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.8666509999999999</v>
+        <v>0.8844070000000001</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.074295</v>
+        <v>0.07581699999999991</v>
       </c>
     </row>
     <row r="16">
@@ -2943,22 +2943,22 @@
         <v>2</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.831483</v>
+        <v>0.852951</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.579431</v>
+        <v>0.594391</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.2520519999999999</v>
+        <v>0.25856</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.942373</v>
+        <v>0.960427</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.865663</v>
+        <v>0.882247</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.07671000000000006</v>
+        <v>0.07818000000000003</v>
       </c>
     </row>
   </sheetData>
@@ -4841,10 +4841,10 @@
         <v>0.668708</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.606936</v>
+        <v>0.613865</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.55731</v>
+        <v>0.563672</v>
       </c>
       <c r="F53" s="3" t="n">
         <v>0.196734</v>
@@ -4856,10 +4856,10 @@
         <v>0.884888</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>0.877918</v>
+        <v>0.888998</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>0.836772</v>
+        <v>0.847333</v>
       </c>
       <c r="K53" s="3" t="n">
         <v>0.211664</v>
@@ -4876,10 +4876,10 @@
         <v>0.676724</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>0.60326</v>
+        <v>0.612673</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0.56216</v>
+        <v>0.570932</v>
       </c>
       <c r="F54" s="3" t="n">
         <v>0.174001</v>
@@ -4891,10 +4891,10 @@
         <v>0.8922870000000001</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>0.873841</v>
+        <v>0.889037</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>0.840377</v>
+        <v>0.8549909999999999</v>
       </c>
       <c r="K54" s="3" t="n">
         <v>0.187696</v>
@@ -4911,10 +4911,10 @@
         <v>0.683503</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>0.600584</v>
+        <v>0.611262</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.566968</v>
+        <v>0.577049</v>
       </c>
       <c r="F55" s="3" t="n">
         <v>0.150377</v>
@@ -4926,10 +4926,10 @@
         <v>0.897388</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>0.870738</v>
+        <v>0.887954</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>0.843601</v>
+        <v>0.860281</v>
       </c>
       <c r="K55" s="3" t="n">
         <v>0.162647</v>
@@ -4946,10 +4946,10 @@
         <v>0.689101</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>0.598208</v>
+        <v>0.609647</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.571229</v>
+        <v>0.582152</v>
       </c>
       <c r="F56" s="3" t="n">
         <v>0.126609</v>
@@ -4961,10 +4961,10 @@
         <v>0.902935</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>0.870319</v>
+        <v>0.888622</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>0.848043</v>
+        <v>0.865878</v>
       </c>
       <c r="K56" s="3" t="n">
         <v>0.137167</v>
@@ -4981,10 +4981,10 @@
         <v>0.693543</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>0.595813</v>
+        <v>0.607845</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0.574761</v>
+        <v>0.586368</v>
       </c>
       <c r="F57" s="3" t="n">
         <v>0.103819</v>
@@ -4996,10 +4996,10 @@
         <v>0.906855</v>
       </c>
       <c r="I57" s="3" t="n">
-        <v>0.869456</v>
+        <v>0.888306</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>0.851382</v>
+        <v>0.869839</v>
       </c>
       <c r="K57" s="3" t="n">
         <v>0.112386</v>
@@ -5016,10 +5016,10 @@
         <v>0.697065</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>0.593449</v>
+        <v>0.6061609999999999</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.57766</v>
+        <v>0.5900339999999999</v>
       </c>
       <c r="F58" s="3" t="n">
         <v>0.083385</v>
@@ -5031,10 +5031,10 @@
         <v>0.910137</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>0.868904</v>
+        <v>0.888008</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>0.854367</v>
+        <v>0.873152</v>
       </c>
       <c r="K58" s="3" t="n">
         <v>0.08956</v>
@@ -5051,10 +5051,10 @@
         <v>0.6996019999999999</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>0.591014</v>
+        <v>0.604614</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0.5798219999999999</v>
+        <v>0.5931650000000001</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>0.066395</v>
@@ -5066,10 +5066,10 @@
         <v>0.912838</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>0.868466</v>
+        <v>0.8876810000000001</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>0.856957</v>
+        <v>0.875918</v>
       </c>
       <c r="K59" s="3" t="n">
         <v>0.06979100000000001</v>
@@ -5086,10 +5086,10 @@
         <v>0.701669</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>0.588936</v>
+        <v>0.603365</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.581641</v>
+        <v>0.5958909999999999</v>
       </c>
       <c r="F60" s="3" t="n">
         <v>0.052954</v>
@@ -5101,10 +5101,10 @@
         <v>0.914806</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>0.867798</v>
+        <v>0.886921</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>0.858953</v>
+        <v>0.877881</v>
       </c>
       <c r="K60" s="3" t="n">
         <v>0.05362</v>
@@ -5121,10 +5121,10 @@
         <v>0.703674</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>0.5873620000000001</v>
+        <v>0.602426</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.583438</v>
+        <v>0.598401</v>
       </c>
       <c r="F61" s="3" t="n">
         <v>0.042558</v>
@@ -5136,10 +5136,10 @@
         <v>0.916965</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>0.86783</v>
+        <v>0.886856</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>0.861187</v>
+        <v>0.880067</v>
       </c>
       <c r="K61" s="3" t="n">
         <v>0.040955</v>
@@ -5156,10 +5156,10 @@
         <v>0.705654</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>0.586135</v>
+        <v>0.601593</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.58523</v>
+        <v>0.600665</v>
       </c>
       <c r="F62" s="3" t="n">
         <v>0.034664</v>
@@ -5171,10 +5171,10 @@
         <v>0.918532</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>0.867586</v>
+        <v>0.886451</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>0.8629019999999999</v>
+        <v>0.8816659999999999</v>
       </c>
       <c r="K62" s="3" t="n">
         <v>0.031309</v>
@@ -5191,10 +5191,10 @@
         <v>0.70778</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>0.585319</v>
+        <v>0.601001</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.587154</v>
+        <v>0.602885</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>0.028742</v>
@@ -5206,10 +5206,10 @@
         <v>0.919894</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>0.867421</v>
+        <v>0.8861</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>0.864447</v>
+        <v>0.883062</v>
       </c>
       <c r="K63" s="3" t="n">
         <v>0.024058</v>
@@ -5226,10 +5226,10 @@
         <v>0.7096789999999999</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>0.584596</v>
+        <v>0.600359</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.588893</v>
+        <v>0.604772</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>0.02431</v>
@@ -5241,10 +5241,10 @@
         <v>0.9209889999999999</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>0.867236</v>
+        <v>0.885675</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>0.865754</v>
+        <v>0.884161</v>
       </c>
       <c r="K64" s="3" t="n">
         <v>0.018627</v>
@@ -5261,10 +5261,10 @@
         <v>0.71128</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>0.583907</v>
+        <v>0.599696</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.590386</v>
+        <v>0.6063499999999999</v>
       </c>
       <c r="F65" s="3" t="n">
         <v>0.020964</v>
@@ -5276,10 +5276,10 @@
         <v>0.921251</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>0.8663729999999999</v>
+        <v>0.884593</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>0.866283</v>
+        <v>0.884501</v>
       </c>
       <c r="K65" s="3" t="n">
         <v>0.014547</v>
@@ -5296,10 +5296,10 @@
         <v>0.712542</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0.58322</v>
+        <v>0.598958</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.591595</v>
+        <v>0.60756</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>0.018384</v>
@@ -5311,10 +5311,10 @@
         <v>0.922529</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>0.866834</v>
+        <v>0.884827</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>0.867769</v>
+        <v>0.885781</v>
       </c>
       <c r="K66" s="3" t="n">
         <v>0.011461</v>
@@ -5331,10 +5331,10 @@
         <v>0.713441</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0.582515</v>
+        <v>0.598167</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.5925010000000001</v>
+        <v>0.608421</v>
       </c>
       <c r="F67" s="3" t="n">
         <v>0.016309</v>
@@ -5346,10 +5346,10 @@
         <v>0.923052</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>0.8666509999999999</v>
+        <v>0.8844070000000001</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>0.868542</v>
+        <v>0.886337</v>
       </c>
       <c r="K67" s="3" t="n">
         <v>0.009109000000000001</v>
@@ -5366,10 +5366,10 @@
         <v>0.714191</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>0.581972</v>
+        <v>0.59751</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.5932770000000001</v>
+        <v>0.609116</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>0.014499</v>
@@ -5381,10 +5381,10 @@
         <v>0.923462</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>0.866506</v>
+        <v>0.884015</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>0.869205</v>
+        <v>0.886769</v>
       </c>
       <c r="K68" s="3" t="n">
         <v>0.007301</v>
@@ -5401,10 +5401,10 @@
         <v>0.714566</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0.581396</v>
+        <v>0.596819</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0.593737</v>
+        <v>0.609487</v>
       </c>
       <c r="F69" s="3" t="n">
         <v>0.012699</v>
@@ -5416,10 +5416,10 @@
         <v>0.9237069999999999</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>0.866335</v>
+        <v>0.8836310000000001</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>0.869707</v>
+        <v>0.88707</v>
       </c>
       <c r="K69" s="3" t="n">
         <v>0.005897</v>
@@ -5436,10 +5436,10 @@
         <v>0.714557</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>0.580783</v>
+        <v>0.596055</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.593874</v>
+        <v>0.60949</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>0.010644</v>
@@ -5451,10 +5451,10 @@
         <v>0.923589</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>0.865917</v>
+        <v>0.882962</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>0.86986</v>
+        <v>0.886982</v>
       </c>
       <c r="K70" s="3" t="n">
         <v>0.004797</v>
@@ -5471,10 +5471,10 @@
         <v>0.714166</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>0.580128</v>
+        <v>0.595247</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.593686</v>
+        <v>0.609158</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>0.008364</v>
@@ -5486,10 +5486,10 @@
         <v>0.9236529999999999</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>0.865821</v>
+        <v>0.882633</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>0.870177</v>
+        <v>0.887074</v>
       </c>
       <c r="K71" s="3" t="n">
         <v>0.003927</v>
@@ -5506,10 +5506,10 @@
         <v>0.713407</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>0.579431</v>
+        <v>0.594391</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.593186</v>
+        <v>0.608502</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>0.006366</v>
@@ -5521,10 +5521,10 @@
         <v>0.923548</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>0.865663</v>
+        <v>0.882247</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>0.870327</v>
+        <v>0.887</v>
       </c>
       <c r="K72" s="3" t="n">
         <v>0.003235</v>

</xml_diff>